<commit_message>
17-08-2026-added wait in Base Updated pageutility
</commit_message>
<xml_diff>
--- a/7RmartSupermarket/src/test/resources/TestDataSample.xlsx
+++ b/7RmartSupermarket/src/test/resources/TestDataSample.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\urmil\eclipse-workspace\7RmartSupermarket\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\urmil\git\MainProjectRepo\7RmartSupermarket\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7721E4C-D4D8-463A-A16D-2CB061491A32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{742E8732-3E4C-49FC-964C-3C824AA40649}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="6" xr2:uid="{8458BAAF-9972-4B30-959C-8E3E9DD375A4}"/>
   </bookViews>
@@ -177,7 +177,7 @@
     <t>12/35,xyz Street,Miami,US</t>
   </si>
   <si>
-    <t>Johns</t>
+    <t>JohnJohny</t>
   </si>
 </sst>
 </file>

</xml_diff>